<commit_message>
multiple changes, debug, default values
</commit_message>
<xml_diff>
--- a/calibration_file/Picarro_results.xlsx
+++ b/calibration_file/Picarro_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruz\Documents\SENSE\horstberry\calibration_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58DE8A8-7279-4366-A836-7C31B4693834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AD7721-EA47-4D33-9929-8C55DCF32E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{B5A3D68D-1C30-46F7-B4F7-AD0109B1ADD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5A3D68D-1C30-46F7-B4F7-AD0109B1ADD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="19">
   <si>
     <t>Gas</t>
   </si>
@@ -93,14 +93,32 @@
     <t>CH4_100ppm_bag_1</t>
   </si>
   <si>
-    <t>CH4_100ppm_bag2</t>
+    <t>CH4_50ppm</t>
+  </si>
+  <si>
+    <t>Picarro</t>
+  </si>
+  <si>
+    <t>RIVER</t>
+  </si>
+  <si>
+    <t>SOIL</t>
+  </si>
+  <si>
+    <t>HP_CH4 (Not suited for our concentration range)</t>
+  </si>
+  <si>
+    <t>CH4_100ppm_bag_2</t>
+  </si>
+  <si>
+    <t>CO2_100_ppm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,12 +133,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -519,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{137ABA74-D92F-4C82-9251-F3C8479DC3F0}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
@@ -529,10 +541,11 @@
     <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -557,10 +570,16 @@
       <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -583,10 +602,14 @@
       <c r="H2" s="1">
         <v>0.189</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -609,10 +632,14 @@
       <c r="H3" s="1">
         <v>0.19</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -635,8 +662,12 @@
       <c r="H4" s="1">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -661,8 +692,12 @@
       <c r="H5" s="1">
         <v>0.09</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -687,8 +722,12 @@
       <c r="H6" s="1">
         <v>0.63</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -713,8 +752,12 @@
       <c r="H7" s="1">
         <v>0.67</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -739,8 +782,12 @@
       <c r="H8" s="1">
         <v>0.69</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -765,8 +812,12 @@
       <c r="H9" s="1">
         <v>0.14000000000000001</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -791,8 +842,14 @@
       <c r="H10" s="1">
         <v>0.54</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="1">
+        <v>83.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -817,8 +874,12 @@
       <c r="H11" s="1">
         <v>0.53</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -843,10 +904,14 @@
       <c r="H12" s="1">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B13" s="1">
         <v>1</v>
@@ -869,10 +934,14 @@
       <c r="H13" s="1">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1">
         <v>2</v>
@@ -895,31 +964,151 @@
       <c r="H14" s="1">
         <v>0.56999999999999995</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="I14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1">
+        <v>100</v>
+      </c>
+      <c r="D15" s="1">
+        <v>92.08</v>
+      </c>
+      <c r="E15" s="1">
+        <v>-37.799999999999997</v>
+      </c>
+      <c r="F15" s="1">
+        <v>17.27</v>
+      </c>
+      <c r="G15" s="1">
+        <v>-922.8</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1">
+        <v>26.5</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="1">
+        <v>8.6999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>100</v>
+      </c>
+      <c r="D17" s="1">
+        <v>89.9</v>
+      </c>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1">
+        <v>23.5</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="1">
+        <v>75.546999999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <v>100</v>
+      </c>
+      <c r="D18" s="1">
+        <v>91.5</v>
+      </c>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1">
+        <v>29</v>
+      </c>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1">
+        <v>0.74</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="1">
+        <v>76.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="2">
-        <v>3</v>
-      </c>
-      <c r="C15" s="2">
-        <v>100</v>
-      </c>
-      <c r="D15" s="2">
-        <v>92.08</v>
-      </c>
-      <c r="E15" s="2">
-        <v>-37.799999999999997</v>
-      </c>
-      <c r="F15" s="2">
-        <v>17.27</v>
-      </c>
-      <c r="G15" s="2">
-        <v>-922.8</v>
-      </c>
-      <c r="H15" s="2">
-        <v>0.56999999999999995</v>
+      <c r="B19" s="2">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2">
+        <v>50</v>
+      </c>
+      <c r="D19" s="2">
+        <v>48.4</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2">
+        <v>13</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2">
+        <v>0.61</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="2">
+        <v>43.354999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>